<commit_message>
add disableAutoDeploy on vercel
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Name</t>
   </si>
@@ -22,13 +22,19 @@
     <t>Tagged</t>
   </si>
   <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>eio98</t>
+  </si>
+  <si>
     <t>[53] Baeju Kael</t>
   </si>
   <si>
-    <t>-1 Jele Lukjaotak ห้ามเลื่อนยศ</t>
-  </si>
-  <si>
-    <t>[88] Cocoa ท้ายร้านเหล้า</t>
+    <t>khanison18</t>
+  </si>
+  <si>
+    <t>coco_sleepcold</t>
   </si>
   <si>
     <t>nxtthawa_t</t>
@@ -41,9 +47,6 @@
   </si>
   <si>
     <t>bxby_cat._</t>
-  </si>
-  <si>
-    <t>khanison18</t>
   </si>
   <si>
     <t>emnjett</t>
@@ -474,14 +477,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="3" width="10" customWidth="1"/>
+    <col min="2" max="4" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -491,98 +494,125 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2">
+        <v>46</v>
+      </c>
+      <c r="C2">
+        <v>104</v>
+      </c>
+      <c r="D2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
         <v>34</v>
       </c>
-      <c r="C2">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3">
-        <v>44</v>
-      </c>
       <c r="C3">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+      <c r="D3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4">
+        <v>36</v>
+      </c>
+      <c r="C4">
+        <v>81</v>
+      </c>
+      <c r="D4">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
         <v>92</v>
       </c>
-      <c r="C4">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
+      <c r="C5">
+        <v>112</v>
+      </c>
+      <c r="D5">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
         <v>32</v>
       </c>
-      <c r="C5">
+      <c r="C6">
         <v>142</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6">
+      <c r="D6">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
         <v>97</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>158</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
+      <c r="D7">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
         <v>52</v>
       </c>
-      <c r="C7">
+      <c r="C8">
         <v>48</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="D8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
         <v>9</v>
       </c>
-      <c r="B8">
-        <v>9</v>
-      </c>
-      <c r="C8">
+      <c r="C9">
         <v>64</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>36</v>
-      </c>
-      <c r="C9">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>4</v>
@@ -590,10 +620,13 @@
       <c r="C10">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>71</v>
@@ -601,10 +634,13 @@
       <c r="C11">
         <v>167</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>19</v>
@@ -612,10 +648,13 @@
       <c r="C12">
         <v>45</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>21</v>
@@ -623,10 +662,13 @@
       <c r="C13">
         <v>37</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -634,10 +676,13 @@
       <c r="C14">
         <v>17</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -645,10 +690,13 @@
       <c r="C15">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>5</v>
@@ -656,10 +704,13 @@
       <c r="C16">
         <v>26</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>5</v>
@@ -667,10 +718,13 @@
       <c r="C17">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>6</v>
@@ -678,10 +732,13 @@
       <c r="C18">
         <v>142</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>16</v>
@@ -689,10 +746,13 @@
       <c r="C19">
         <v>74</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B20">
         <v>4</v>
@@ -700,10 +760,13 @@
       <c r="C20">
         <v>24</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B21">
         <v>20</v>
@@ -711,10 +774,13 @@
       <c r="C21">
         <v>31</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -722,10 +788,13 @@
       <c r="C22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B23">
         <v>2</v>
@@ -733,10 +802,13 @@
       <c r="C23">
         <v>5</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D23">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -744,10 +816,13 @@
       <c r="C24">
         <v>7</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D24">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -755,10 +830,13 @@
       <c r="C25">
         <v>18</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -766,15 +844,21 @@
       <c r="C26">
         <v>3</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
       <c r="C27">
+        <v>20</v>
+      </c>
+      <c r="D27">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
load Nicename And Log notFound
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -25,82 +25,82 @@
     <t>Total</t>
   </si>
   <si>
-    <t>eio98</t>
-  </si>
-  <si>
     <t>[53] Baeju Kael</t>
   </si>
   <si>
-    <t>khanison18</t>
-  </si>
-  <si>
-    <t>coco_sleepcold</t>
-  </si>
-  <si>
-    <t>nxtthawa_t</t>
+    <t>-1 Jele Lukjaotak ห้ามเลื่อนยศ</t>
+  </si>
+  <si>
+    <t>[09] Lauren Rokashi</t>
+  </si>
+  <si>
+    <t>[88] Cocoa ท้ายร้านเหล้า</t>
+  </si>
+  <si>
+    <t>[03] Simon Miracle</t>
   </si>
   <si>
     <t>lone_z</t>
   </si>
   <si>
-    <t>game7820</t>
-  </si>
-  <si>
-    <t>bxby_cat._</t>
-  </si>
-  <si>
-    <t>emnjett</t>
-  </si>
-  <si>
-    <t>skygo._ap</t>
-  </si>
-  <si>
-    <t>avanaja</t>
-  </si>
-  <si>
-    <t>noname141767</t>
-  </si>
-  <si>
-    <t>zimbaraone</t>
+    <t>[89]Game Harrington</t>
+  </si>
+  <si>
+    <t>[24] Lilin Miller</t>
+  </si>
+  <si>
+    <t>[84]  Yoko Mehay</t>
+  </si>
+  <si>
+    <t>[90]Sky Lukjaotak</t>
+  </si>
+  <si>
+    <t>[06]Kanomthom Jaa</t>
+  </si>
+  <si>
+    <t>[77] Name Aribrabra</t>
+  </si>
+  <si>
+    <t>[66]Del Mirano</t>
   </si>
   <si>
     <t>ta099561</t>
   </si>
   <si>
-    <t>on_name</t>
-  </si>
-  <si>
-    <t>lil.chag.</t>
-  </si>
-  <si>
-    <t>time_walker1764</t>
-  </si>
-  <si>
-    <t>hyong15a</t>
-  </si>
-  <si>
-    <t>maxx7767</t>
-  </si>
-  <si>
-    <t>shoppymaibok3145</t>
-  </si>
-  <si>
-    <t>franklampard0035</t>
-  </si>
-  <si>
-    <t>mumi0171</t>
-  </si>
-  <si>
-    <t>dan0772</t>
-  </si>
-  <si>
-    <t>_newwys</t>
+    <t>[02]JOHN LUKJAOTAK</t>
+  </si>
+  <si>
+    <t>[058] Loid Sunset</t>
+  </si>
+  <si>
+    <t>[21] Time Walker เคาะจาน !!</t>
+  </si>
+  <si>
+    <t>[015] Hyong Lukjaotak</t>
+  </si>
+  <si>
+    <t>[56] Max TuaraiSpicy ท้ายKFC</t>
+  </si>
+  <si>
+    <t>[57]shoppy maibok</t>
+  </si>
+  <si>
+    <t>[05] Blxck Noris</t>
+  </si>
+  <si>
+    <t>[77] New Mumi</t>
+  </si>
+  <si>
+    <t>[008]DanNew Uzi</t>
+  </si>
+  <si>
+    <t>[48] Newwy Jawatpa</t>
   </si>
   <si>
     <t>mna5555za</t>
   </si>
   <si>
-    <t>dionfunyup</t>
+    <t>[44]Dion Funyup</t>
   </si>
 </sst>
 </file>
@@ -503,13 +503,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="C2">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="D2">
-        <v>150</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -517,13 +517,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C3">
-        <v>60</v>
+        <v>104</v>
       </c>
       <c r="D3">
-        <v>94</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>